<commit_message>
Added dishwashers, refrigerators, and air conditioners for Bosch
</commit_message>
<xml_diff>
--- a/reports/BSH_Detayli_Fiyat_Raporu.xlsx
+++ b/reports/BSH_Detayli_Fiyat_Raporu.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="171">
   <si>
     <t>Marka</t>
   </si>
@@ -40,9 +40,111 @@
     <t>Bosch</t>
   </si>
   <si>
+    <t>Bulaşık Makinesi</t>
+  </si>
+  <si>
+    <t>Buzdolabı</t>
+  </si>
+  <si>
+    <t>Klima</t>
+  </si>
+  <si>
     <t>Çamaşır Makinesi</t>
   </si>
   <si>
+    <t>SMV4IMX62T</t>
+  </si>
+  <si>
+    <t>SMS6EMI63T</t>
+  </si>
+  <si>
+    <t>SMP6ENC60T</t>
+  </si>
+  <si>
+    <t>SMS6ENW60T</t>
+  </si>
+  <si>
+    <t>SMS6ENY60T</t>
+  </si>
+  <si>
+    <t>SMS6ENB60T</t>
+  </si>
+  <si>
+    <t>SMS4HMY62T</t>
+  </si>
+  <si>
+    <t>SMS6ECI83T</t>
+  </si>
+  <si>
+    <t>SMI6EKS81T</t>
+  </si>
+  <si>
+    <t>SMV6ECX86Q</t>
+  </si>
+  <si>
+    <t>SMS8YDI82T</t>
+  </si>
+  <si>
+    <t>SMI8ZDS81T</t>
+  </si>
+  <si>
+    <t>KGN76CXE0N</t>
+  </si>
+  <si>
+    <t>KGP76AWC0N</t>
+  </si>
+  <si>
+    <t>KDN86AWE1N</t>
+  </si>
+  <si>
+    <t>KGN86AID2N</t>
+  </si>
+  <si>
+    <t>KGA76PIE0N</t>
+  </si>
+  <si>
+    <t>KGP76AIC0N</t>
+  </si>
+  <si>
+    <t>KDN86AID1N</t>
+  </si>
+  <si>
+    <t>KGP86FWC0N</t>
+  </si>
+  <si>
+    <t>KGP86FIC0N</t>
+  </si>
+  <si>
+    <t>KGP86AXB0N</t>
+  </si>
+  <si>
+    <t>KFN96VPEA</t>
+  </si>
+  <si>
+    <t>KBN96ADD0</t>
+  </si>
+  <si>
+    <t>ASX09VW32N</t>
+  </si>
+  <si>
+    <t>ASX12VW32N</t>
+  </si>
+  <si>
+    <t>ASX12XB32N</t>
+  </si>
+  <si>
+    <t>ASX18VW32N</t>
+  </si>
+  <si>
+    <t>ASX18XB32N</t>
+  </si>
+  <si>
+    <t>ASX24VW32N</t>
+  </si>
+  <si>
+    <t>WGA254A0TR</t>
+  </si>
+  <si>
     <t>WGK242Z0TR</t>
   </si>
   <si>
@@ -79,6 +181,72 @@
     <t>WGK264ZRTR</t>
   </si>
   <si>
+    <t>Serie 6 Tam Ankastre Bulaşık Makinesi 60 cm</t>
+  </si>
+  <si>
+    <t>Serie 6 Solo Bulaşık Makinesi 60 cm Kolay Temizlenebilir Inox</t>
+  </si>
+  <si>
+    <t>Serie 6 Solo Bulaşık Makinesi 60 cm Kolay Temizlenebilir Siyah Inox</t>
+  </si>
+  <si>
+    <t>Serie 6 Solo Bulaşık Makinesi 60 cm Beyaz</t>
+  </si>
+  <si>
+    <t>Serie 6 Solo Bulaşık Makinesi 60 cm</t>
+  </si>
+  <si>
+    <t>Serie 6 Solo Bulaşık Makinesi 60 cm Siyah</t>
+  </si>
+  <si>
+    <t>Serie 6 Yarı Ankastre Bulaşık Makinesi 60 cm Paslanmaz çelik</t>
+  </si>
+  <si>
+    <t>Serie 8 Solo Bulaşık Makinesi 60 cm Kolay Temizlenebilir Inox</t>
+  </si>
+  <si>
+    <t>Serie 8 Yarı Ankastre Bulaşık Makinesi 60 cm Paslanmaz çelik</t>
+  </si>
+  <si>
+    <t>Serie 6 Alttan Donduruculu Buzdolabı 186 x 75 cm Parmak izi bırakmayan siyah inoks</t>
+  </si>
+  <si>
+    <t>Serie 8 Alttan Donduruculu Buzdolabı 186 x 75 cm Beyaz, Total No Frost</t>
+  </si>
+  <si>
+    <t>Serie 6 Üstten Donduruculu Buzdolabı 186 x 86 cm Beyaz, Total No Frost</t>
+  </si>
+  <si>
+    <t>Serie 6 Alttan Donduruculu Buzdolabı 186 x 86 cm Paslanmaz çelik</t>
+  </si>
+  <si>
+    <t>Serie 8 Alttan Donduruculu Buzdolabı 186 x 75 cm Paslanmaz çelik</t>
+  </si>
+  <si>
+    <t>Serie 6 Üstten Donduruculu Buzdolabı 186 x 86 cm Paslanmaz çelik</t>
+  </si>
+  <si>
+    <t>Serie 8 Alttan Donduruculu Buzdolabı 186 x 86 cm Beyaz, Total No Frost</t>
+  </si>
+  <si>
+    <t>Serie 8 Alttan Donduruculu Buzdolabı 186 x 86 cm Paslanmaz çelik</t>
+  </si>
+  <si>
+    <t>Serie 8 Alttan Donduruculu Buzdolabı 186 x 86 cm Parmak izi bırakmayan siyah inoks</t>
+  </si>
+  <si>
+    <t>Serie 4 Gardırop Tipi Buzdolabı 183 x 90.5 cm Paslanmaz çelik</t>
+  </si>
+  <si>
+    <t>Serie 6 Alttan Donduruculu Ankastre Buzdolabı 193.5 x 70.8 cm softClosing Düz Menteşe</t>
+  </si>
+  <si>
+    <t>Klima, Ev Tipi</t>
+  </si>
+  <si>
+    <t>Bosch 10 kg 1200 Devir Çamaşır Makinesi</t>
+  </si>
+  <si>
     <t>Serie 6 Çamaşır Makinesi 9 kg maks. 1200 dev./dak.</t>
   </si>
   <si>
@@ -106,40 +274,259 @@
     <t>Stokta Var</t>
   </si>
   <si>
+    <t>2026-07-01 17:19:38</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:34</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:19:44</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:24</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:19:54</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:25</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:19:40</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:19:46</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:20:00</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:29</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:33</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:36</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:19:59</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:27</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:19:50</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:41</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:19:52</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:31</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:19:42</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:42</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:19:56</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:22</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:19:48</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:38</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:25:02</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:48</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:50</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:53</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:58</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:25:04</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:52</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:25:08</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:47</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:25:06</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:25:00</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:55</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:20:11</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:25:19</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:20:13</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:25:13</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:20:16</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:25:21</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:20:17</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:25:12</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:20:08</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:25:17</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:20:10</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:25:15</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:16:14</t>
+  </si>
+  <si>
     <t>2026-07-01 16:55:44</t>
   </si>
   <si>
+    <t>2026-07-01 17:19:28</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:12</t>
+  </si>
+  <si>
     <t>2026-07-01 16:55:50</t>
   </si>
   <si>
+    <t>2026-07-01 17:19:23</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:11</t>
+  </si>
+  <si>
     <t>2026-07-01 16:55:59</t>
   </si>
   <si>
+    <t>2026-07-01 17:19:30</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:09</t>
+  </si>
+  <si>
     <t>2026-07-01 16:55:46</t>
   </si>
   <si>
+    <t>2026-07-01 17:19:17</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:04</t>
+  </si>
+  <si>
     <t>2026-07-01 16:56:02</t>
   </si>
   <si>
+    <t>2026-07-01 17:19:32</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:00</t>
+  </si>
+  <si>
     <t>2026-07-01 16:55:49</t>
   </si>
   <si>
+    <t>2026-07-01 17:19:19</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:16</t>
+  </si>
+  <si>
     <t>2026-07-01 16:55:57</t>
   </si>
   <si>
+    <t>2026-07-01 17:19:26</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:02</t>
+  </si>
+  <si>
     <t>2026-07-01 16:55:47</t>
   </si>
   <si>
+    <t>2026-07-01 17:19:33</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:18</t>
+  </si>
+  <si>
     <t>2026-07-01 16:55:55</t>
   </si>
   <si>
+    <t>2026-07-01 17:19:14</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:06</t>
+  </si>
+  <si>
     <t>2026-07-01 16:56:00</t>
   </si>
   <si>
+    <t>2026-07-01 17:19:24</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:23:58</t>
+  </si>
+  <si>
     <t>2026-07-01 16:55:53</t>
   </si>
   <si>
+    <t>2026-07-01 17:19:21</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:14</t>
+  </si>
+  <si>
     <t>2026-07-01 16:55:52</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:19:16</t>
+  </si>
+  <si>
+    <t>2026-07-01 17:24:07</t>
   </si>
 </sst>
 </file>
@@ -497,7 +884,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -531,19 +918,19 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>55</v>
       </c>
       <c r="E2">
-        <v>44510</v>
+        <v>44350</v>
       </c>
       <c r="F2" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="G2" t="s">
-        <v>30</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -554,19 +941,19 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="E3">
-        <v>46040</v>
+        <v>44350</v>
       </c>
       <c r="F3" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="G3" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -577,19 +964,19 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="E4">
-        <v>46210</v>
+        <v>44430</v>
       </c>
       <c r="F4" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="G4" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -600,19 +987,19 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="E5">
-        <v>46440</v>
+        <v>44430</v>
       </c>
       <c r="F5" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="G5" t="s">
-        <v>33</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -623,19 +1010,19 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="E6">
-        <v>46560</v>
+        <v>45080</v>
       </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="G6" t="s">
-        <v>34</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -649,16 +1036,16 @@
         <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="E7">
-        <v>47150</v>
+        <v>45080</v>
       </c>
       <c r="F7" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="G7" t="s">
-        <v>35</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -672,16 +1059,16 @@
         <v>15</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="E8">
-        <v>48310</v>
+        <v>47010</v>
       </c>
       <c r="F8" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="G8" t="s">
-        <v>36</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -695,16 +1082,16 @@
         <v>16</v>
       </c>
       <c r="D9" t="s">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="E9">
-        <v>48460</v>
+        <v>47010</v>
       </c>
       <c r="F9" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="G9" t="s">
-        <v>37</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -718,16 +1105,16 @@
         <v>17</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="E10">
-        <v>49700</v>
+        <v>47010</v>
       </c>
       <c r="F10" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="G10" t="s">
-        <v>38</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -738,19 +1125,19 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="E11">
-        <v>51090</v>
+        <v>47010</v>
       </c>
       <c r="F11" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="G11" t="s">
-        <v>39</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -761,19 +1148,19 @@
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D12" t="s">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="E12">
-        <v>52660</v>
+        <v>47010</v>
       </c>
       <c r="F12" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="G12" t="s">
-        <v>40</v>
+        <v>96</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -784,19 +1171,1698 @@
         <v>8</v>
       </c>
       <c r="C13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13">
+        <v>47010</v>
+      </c>
+      <c r="F13" t="s">
+        <v>85</v>
+      </c>
+      <c r="G13" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" t="s">
+        <v>59</v>
+      </c>
+      <c r="E14">
+        <v>51300</v>
+      </c>
+      <c r="F14" t="s">
+        <v>85</v>
+      </c>
+      <c r="G14" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" t="s">
+        <v>59</v>
+      </c>
+      <c r="E15">
+        <v>51300</v>
+      </c>
+      <c r="F15" t="s">
+        <v>85</v>
+      </c>
+      <c r="G15" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" t="s">
+        <v>56</v>
+      </c>
+      <c r="E16">
+        <v>59970</v>
+      </c>
+      <c r="F16" t="s">
+        <v>85</v>
+      </c>
+      <c r="G16" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17">
+        <v>59970</v>
+      </c>
+      <c r="F17" t="s">
+        <v>85</v>
+      </c>
+      <c r="G17" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" t="s">
         <v>20</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D18" t="s">
+        <v>61</v>
+      </c>
+      <c r="E18">
+        <v>62580</v>
+      </c>
+      <c r="F18" t="s">
+        <v>85</v>
+      </c>
+      <c r="G18" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" t="s">
+        <v>61</v>
+      </c>
+      <c r="E19">
+        <v>62580</v>
+      </c>
+      <c r="F19" t="s">
+        <v>85</v>
+      </c>
+      <c r="G19" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
+        <v>21</v>
+      </c>
+      <c r="D20" t="s">
+        <v>55</v>
+      </c>
+      <c r="E20">
+        <v>63200</v>
+      </c>
+      <c r="F20" t="s">
+        <v>85</v>
+      </c>
+      <c r="G20" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" t="s">
+        <v>7</v>
+      </c>
+      <c r="B21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" t="s">
+        <v>21</v>
+      </c>
+      <c r="D21" t="s">
+        <v>55</v>
+      </c>
+      <c r="E21">
+        <v>63200</v>
+      </c>
+      <c r="F21" t="s">
+        <v>85</v>
+      </c>
+      <c r="G21" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" t="s">
+        <v>7</v>
+      </c>
+      <c r="B22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" t="s">
+        <v>22</v>
+      </c>
+      <c r="D22" t="s">
+        <v>62</v>
+      </c>
+      <c r="E22">
+        <v>66470</v>
+      </c>
+      <c r="F22" t="s">
+        <v>85</v>
+      </c>
+      <c r="G22" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" t="s">
+        <v>22</v>
+      </c>
+      <c r="D23" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23">
+        <v>66470</v>
+      </c>
+      <c r="F23" t="s">
+        <v>85</v>
+      </c>
+      <c r="G23" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" t="s">
+        <v>23</v>
+      </c>
+      <c r="D24" t="s">
+        <v>63</v>
+      </c>
+      <c r="E24">
+        <v>81510</v>
+      </c>
+      <c r="F24" t="s">
+        <v>85</v>
+      </c>
+      <c r="G24" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" t="s">
+        <v>23</v>
+      </c>
+      <c r="D25" t="s">
+        <v>63</v>
+      </c>
+      <c r="E25">
+        <v>81510</v>
+      </c>
+      <c r="F25" t="s">
+        <v>85</v>
+      </c>
+      <c r="G25" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26" t="s">
+        <v>64</v>
+      </c>
+      <c r="E26">
+        <v>87390</v>
+      </c>
+      <c r="F26" t="s">
+        <v>85</v>
+      </c>
+      <c r="G26" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" t="s">
+        <v>25</v>
+      </c>
+      <c r="D27" t="s">
+        <v>65</v>
+      </c>
+      <c r="E27">
+        <v>87890</v>
+      </c>
+      <c r="F27" t="s">
+        <v>85</v>
+      </c>
+      <c r="G27" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" t="s">
+        <v>66</v>
+      </c>
+      <c r="E28">
+        <v>88600</v>
+      </c>
+      <c r="F28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G28" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" t="s">
+        <v>27</v>
+      </c>
+      <c r="D29" t="s">
+        <v>67</v>
+      </c>
+      <c r="E29">
+        <v>94490</v>
+      </c>
+      <c r="F29" t="s">
+        <v>85</v>
+      </c>
+      <c r="G29" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" t="s">
         <v>28</v>
       </c>
-      <c r="E13">
+      <c r="D30" t="s">
+        <v>68</v>
+      </c>
+      <c r="E30">
+        <v>94890</v>
+      </c>
+      <c r="F30" t="s">
+        <v>85</v>
+      </c>
+      <c r="G30" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" t="s">
+        <v>7</v>
+      </c>
+      <c r="B31" t="s">
+        <v>9</v>
+      </c>
+      <c r="C31" t="s">
+        <v>29</v>
+      </c>
+      <c r="D31" t="s">
+        <v>68</v>
+      </c>
+      <c r="E31">
+        <v>95390</v>
+      </c>
+      <c r="F31" t="s">
+        <v>85</v>
+      </c>
+      <c r="G31" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" t="s">
+        <v>7</v>
+      </c>
+      <c r="B32" t="s">
+        <v>9</v>
+      </c>
+      <c r="C32" t="s">
+        <v>30</v>
+      </c>
+      <c r="D32" t="s">
+        <v>69</v>
+      </c>
+      <c r="E32">
+        <v>96750</v>
+      </c>
+      <c r="F32" t="s">
+        <v>85</v>
+      </c>
+      <c r="G32" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" t="s">
+        <v>7</v>
+      </c>
+      <c r="B33" t="s">
+        <v>9</v>
+      </c>
+      <c r="C33" t="s">
+        <v>31</v>
+      </c>
+      <c r="D33" t="s">
+        <v>70</v>
+      </c>
+      <c r="E33">
+        <v>99790</v>
+      </c>
+      <c r="F33" t="s">
+        <v>85</v>
+      </c>
+      <c r="G33" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" t="s">
+        <v>7</v>
+      </c>
+      <c r="B34" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" t="s">
+        <v>32</v>
+      </c>
+      <c r="D34" t="s">
+        <v>71</v>
+      </c>
+      <c r="E34">
+        <v>105790</v>
+      </c>
+      <c r="F34" t="s">
+        <v>85</v>
+      </c>
+      <c r="G34" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" t="s">
+        <v>7</v>
+      </c>
+      <c r="B35" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" t="s">
+        <v>33</v>
+      </c>
+      <c r="D35" t="s">
+        <v>72</v>
+      </c>
+      <c r="E35">
+        <v>115290</v>
+      </c>
+      <c r="F35" t="s">
+        <v>85</v>
+      </c>
+      <c r="G35" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" t="s">
+        <v>7</v>
+      </c>
+      <c r="B36" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" t="s">
+        <v>34</v>
+      </c>
+      <c r="D36" t="s">
+        <v>73</v>
+      </c>
+      <c r="E36">
+        <v>122990</v>
+      </c>
+      <c r="F36" t="s">
+        <v>85</v>
+      </c>
+      <c r="G36" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" t="s">
+        <v>7</v>
+      </c>
+      <c r="B37" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" t="s">
+        <v>35</v>
+      </c>
+      <c r="D37" t="s">
+        <v>74</v>
+      </c>
+      <c r="E37">
+        <v>127110</v>
+      </c>
+      <c r="F37" t="s">
+        <v>85</v>
+      </c>
+      <c r="G37" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" t="s">
+        <v>7</v>
+      </c>
+      <c r="B38" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38" t="s">
+        <v>36</v>
+      </c>
+      <c r="D38" t="s">
+        <v>75</v>
+      </c>
+      <c r="E38">
+        <v>45700</v>
+      </c>
+      <c r="F38" t="s">
+        <v>85</v>
+      </c>
+      <c r="G38" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" t="s">
+        <v>7</v>
+      </c>
+      <c r="B39" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" t="s">
+        <v>36</v>
+      </c>
+      <c r="D39" t="s">
+        <v>75</v>
+      </c>
+      <c r="E39">
+        <v>45700</v>
+      </c>
+      <c r="F39" t="s">
+        <v>85</v>
+      </c>
+      <c r="G39" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" t="s">
+        <v>7</v>
+      </c>
+      <c r="B40" t="s">
+        <v>10</v>
+      </c>
+      <c r="C40" t="s">
+        <v>37</v>
+      </c>
+      <c r="D40" t="s">
+        <v>75</v>
+      </c>
+      <c r="E40">
+        <v>50200</v>
+      </c>
+      <c r="F40" t="s">
+        <v>85</v>
+      </c>
+      <c r="G40" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" t="s">
+        <v>7</v>
+      </c>
+      <c r="B41" t="s">
+        <v>10</v>
+      </c>
+      <c r="C41" t="s">
+        <v>37</v>
+      </c>
+      <c r="D41" t="s">
+        <v>75</v>
+      </c>
+      <c r="E41">
+        <v>50200</v>
+      </c>
+      <c r="F41" t="s">
+        <v>85</v>
+      </c>
+      <c r="G41" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" t="s">
+        <v>7</v>
+      </c>
+      <c r="B42" t="s">
+        <v>10</v>
+      </c>
+      <c r="C42" t="s">
+        <v>38</v>
+      </c>
+      <c r="D42" t="s">
+        <v>75</v>
+      </c>
+      <c r="E42">
+        <v>56030</v>
+      </c>
+      <c r="F42" t="s">
+        <v>85</v>
+      </c>
+      <c r="G42" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43" t="s">
+        <v>7</v>
+      </c>
+      <c r="B43" t="s">
+        <v>10</v>
+      </c>
+      <c r="C43" t="s">
+        <v>38</v>
+      </c>
+      <c r="D43" t="s">
+        <v>75</v>
+      </c>
+      <c r="E43">
+        <v>56030</v>
+      </c>
+      <c r="F43" t="s">
+        <v>85</v>
+      </c>
+      <c r="G43" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44" t="s">
+        <v>7</v>
+      </c>
+      <c r="B44" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" t="s">
+        <v>39</v>
+      </c>
+      <c r="D44" t="s">
+        <v>75</v>
+      </c>
+      <c r="E44">
+        <v>70810</v>
+      </c>
+      <c r="F44" t="s">
+        <v>85</v>
+      </c>
+      <c r="G44" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45" t="s">
+        <v>7</v>
+      </c>
+      <c r="B45" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" t="s">
+        <v>39</v>
+      </c>
+      <c r="D45" t="s">
+        <v>75</v>
+      </c>
+      <c r="E45">
+        <v>70810</v>
+      </c>
+      <c r="F45" t="s">
+        <v>85</v>
+      </c>
+      <c r="G45" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
+      <c r="A46" t="s">
+        <v>7</v>
+      </c>
+      <c r="B46" t="s">
+        <v>10</v>
+      </c>
+      <c r="C46" t="s">
+        <v>40</v>
+      </c>
+      <c r="D46" t="s">
+        <v>75</v>
+      </c>
+      <c r="E46">
+        <v>79070</v>
+      </c>
+      <c r="F46" t="s">
+        <v>85</v>
+      </c>
+      <c r="G46" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
+      <c r="A47" t="s">
+        <v>7</v>
+      </c>
+      <c r="B47" t="s">
+        <v>10</v>
+      </c>
+      <c r="C47" t="s">
+        <v>40</v>
+      </c>
+      <c r="D47" t="s">
+        <v>75</v>
+      </c>
+      <c r="E47">
+        <v>79070</v>
+      </c>
+      <c r="F47" t="s">
+        <v>85</v>
+      </c>
+      <c r="G47" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48" t="s">
+        <v>7</v>
+      </c>
+      <c r="B48" t="s">
+        <v>10</v>
+      </c>
+      <c r="C48" t="s">
+        <v>41</v>
+      </c>
+      <c r="D48" t="s">
+        <v>75</v>
+      </c>
+      <c r="E48">
+        <v>85790</v>
+      </c>
+      <c r="F48" t="s">
+        <v>85</v>
+      </c>
+      <c r="G48" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49" t="s">
+        <v>7</v>
+      </c>
+      <c r="B49" t="s">
+        <v>10</v>
+      </c>
+      <c r="C49" t="s">
+        <v>41</v>
+      </c>
+      <c r="D49" t="s">
+        <v>75</v>
+      </c>
+      <c r="E49">
+        <v>85790</v>
+      </c>
+      <c r="F49" t="s">
+        <v>85</v>
+      </c>
+      <c r="G49" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
+      <c r="A50" t="s">
+        <v>7</v>
+      </c>
+      <c r="B50" t="s">
+        <v>11</v>
+      </c>
+      <c r="C50" t="s">
+        <v>42</v>
+      </c>
+      <c r="D50" t="s">
+        <v>76</v>
+      </c>
+      <c r="E50">
+        <v>24500</v>
+      </c>
+      <c r="F50" t="s">
+        <v>85</v>
+      </c>
+      <c r="G50" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
+      <c r="A51" t="s">
+        <v>7</v>
+      </c>
+      <c r="B51" t="s">
+        <v>11</v>
+      </c>
+      <c r="C51" t="s">
+        <v>43</v>
+      </c>
+      <c r="D51" t="s">
+        <v>77</v>
+      </c>
+      <c r="E51">
+        <v>44510</v>
+      </c>
+      <c r="F51" t="s">
+        <v>85</v>
+      </c>
+      <c r="G51" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
+      <c r="A52" t="s">
+        <v>7</v>
+      </c>
+      <c r="B52" t="s">
+        <v>11</v>
+      </c>
+      <c r="C52" t="s">
+        <v>43</v>
+      </c>
+      <c r="D52" t="s">
+        <v>77</v>
+      </c>
+      <c r="E52">
+        <v>44510</v>
+      </c>
+      <c r="F52" t="s">
+        <v>85</v>
+      </c>
+      <c r="G52" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
+      <c r="A53" t="s">
+        <v>7</v>
+      </c>
+      <c r="B53" t="s">
+        <v>11</v>
+      </c>
+      <c r="C53" t="s">
+        <v>43</v>
+      </c>
+      <c r="D53" t="s">
+        <v>77</v>
+      </c>
+      <c r="E53">
+        <v>44510</v>
+      </c>
+      <c r="F53" t="s">
+        <v>85</v>
+      </c>
+      <c r="G53" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
+      <c r="A54" t="s">
+        <v>7</v>
+      </c>
+      <c r="B54" t="s">
+        <v>11</v>
+      </c>
+      <c r="C54" t="s">
+        <v>44</v>
+      </c>
+      <c r="D54" t="s">
+        <v>78</v>
+      </c>
+      <c r="E54">
+        <v>46040</v>
+      </c>
+      <c r="F54" t="s">
+        <v>85</v>
+      </c>
+      <c r="G54" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
+      <c r="A55" t="s">
+        <v>7</v>
+      </c>
+      <c r="B55" t="s">
+        <v>11</v>
+      </c>
+      <c r="C55" t="s">
+        <v>44</v>
+      </c>
+      <c r="D55" t="s">
+        <v>78</v>
+      </c>
+      <c r="E55">
+        <v>46040</v>
+      </c>
+      <c r="F55" t="s">
+        <v>85</v>
+      </c>
+      <c r="G55" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
+      <c r="A56" t="s">
+        <v>7</v>
+      </c>
+      <c r="B56" t="s">
+        <v>11</v>
+      </c>
+      <c r="C56" t="s">
+        <v>44</v>
+      </c>
+      <c r="D56" t="s">
+        <v>78</v>
+      </c>
+      <c r="E56">
+        <v>46040</v>
+      </c>
+      <c r="F56" t="s">
+        <v>85</v>
+      </c>
+      <c r="G56" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
+      <c r="A57" t="s">
+        <v>7</v>
+      </c>
+      <c r="B57" t="s">
+        <v>11</v>
+      </c>
+      <c r="C57" t="s">
+        <v>45</v>
+      </c>
+      <c r="D57" t="s">
+        <v>79</v>
+      </c>
+      <c r="E57">
+        <v>46210</v>
+      </c>
+      <c r="F57" t="s">
+        <v>85</v>
+      </c>
+      <c r="G57" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
+      <c r="A58" t="s">
+        <v>7</v>
+      </c>
+      <c r="B58" t="s">
+        <v>11</v>
+      </c>
+      <c r="C58" t="s">
+        <v>45</v>
+      </c>
+      <c r="D58" t="s">
+        <v>79</v>
+      </c>
+      <c r="E58">
+        <v>46210</v>
+      </c>
+      <c r="F58" t="s">
+        <v>85</v>
+      </c>
+      <c r="G58" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7">
+      <c r="A59" t="s">
+        <v>7</v>
+      </c>
+      <c r="B59" t="s">
+        <v>11</v>
+      </c>
+      <c r="C59" t="s">
+        <v>45</v>
+      </c>
+      <c r="D59" t="s">
+        <v>79</v>
+      </c>
+      <c r="E59">
+        <v>46210</v>
+      </c>
+      <c r="F59" t="s">
+        <v>85</v>
+      </c>
+      <c r="G59" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7">
+      <c r="A60" t="s">
+        <v>7</v>
+      </c>
+      <c r="B60" t="s">
+        <v>11</v>
+      </c>
+      <c r="C60" t="s">
+        <v>46</v>
+      </c>
+      <c r="D60" t="s">
+        <v>80</v>
+      </c>
+      <c r="E60">
+        <v>46440</v>
+      </c>
+      <c r="F60" t="s">
+        <v>85</v>
+      </c>
+      <c r="G60" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7">
+      <c r="A61" t="s">
+        <v>7</v>
+      </c>
+      <c r="B61" t="s">
+        <v>11</v>
+      </c>
+      <c r="C61" t="s">
+        <v>46</v>
+      </c>
+      <c r="D61" t="s">
+        <v>80</v>
+      </c>
+      <c r="E61">
+        <v>46440</v>
+      </c>
+      <c r="F61" t="s">
+        <v>85</v>
+      </c>
+      <c r="G61" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7">
+      <c r="A62" t="s">
+        <v>7</v>
+      </c>
+      <c r="B62" t="s">
+        <v>11</v>
+      </c>
+      <c r="C62" t="s">
+        <v>46</v>
+      </c>
+      <c r="D62" t="s">
+        <v>80</v>
+      </c>
+      <c r="E62">
+        <v>46440</v>
+      </c>
+      <c r="F62" t="s">
+        <v>85</v>
+      </c>
+      <c r="G62" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7">
+      <c r="A63" t="s">
+        <v>7</v>
+      </c>
+      <c r="B63" t="s">
+        <v>11</v>
+      </c>
+      <c r="C63" t="s">
+        <v>47</v>
+      </c>
+      <c r="D63" t="s">
+        <v>80</v>
+      </c>
+      <c r="E63">
+        <v>46560</v>
+      </c>
+      <c r="F63" t="s">
+        <v>85</v>
+      </c>
+      <c r="G63" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7">
+      <c r="A64" t="s">
+        <v>7</v>
+      </c>
+      <c r="B64" t="s">
+        <v>11</v>
+      </c>
+      <c r="C64" t="s">
+        <v>47</v>
+      </c>
+      <c r="D64" t="s">
+        <v>80</v>
+      </c>
+      <c r="E64">
+        <v>46560</v>
+      </c>
+      <c r="F64" t="s">
+        <v>85</v>
+      </c>
+      <c r="G64" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7">
+      <c r="A65" t="s">
+        <v>7</v>
+      </c>
+      <c r="B65" t="s">
+        <v>11</v>
+      </c>
+      <c r="C65" t="s">
+        <v>47</v>
+      </c>
+      <c r="D65" t="s">
+        <v>80</v>
+      </c>
+      <c r="E65">
+        <v>46560</v>
+      </c>
+      <c r="F65" t="s">
+        <v>85</v>
+      </c>
+      <c r="G65" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7">
+      <c r="A66" t="s">
+        <v>7</v>
+      </c>
+      <c r="B66" t="s">
+        <v>11</v>
+      </c>
+      <c r="C66" t="s">
+        <v>48</v>
+      </c>
+      <c r="D66" t="s">
+        <v>81</v>
+      </c>
+      <c r="E66">
+        <v>47150</v>
+      </c>
+      <c r="F66" t="s">
+        <v>85</v>
+      </c>
+      <c r="G66" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7">
+      <c r="A67" t="s">
+        <v>7</v>
+      </c>
+      <c r="B67" t="s">
+        <v>11</v>
+      </c>
+      <c r="C67" t="s">
+        <v>48</v>
+      </c>
+      <c r="D67" t="s">
+        <v>81</v>
+      </c>
+      <c r="E67">
+        <v>47150</v>
+      </c>
+      <c r="F67" t="s">
+        <v>85</v>
+      </c>
+      <c r="G67" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7">
+      <c r="A68" t="s">
+        <v>7</v>
+      </c>
+      <c r="B68" t="s">
+        <v>11</v>
+      </c>
+      <c r="C68" t="s">
+        <v>48</v>
+      </c>
+      <c r="D68" t="s">
+        <v>81</v>
+      </c>
+      <c r="E68">
+        <v>47150</v>
+      </c>
+      <c r="F68" t="s">
+        <v>85</v>
+      </c>
+      <c r="G68" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7">
+      <c r="A69" t="s">
+        <v>7</v>
+      </c>
+      <c r="B69" t="s">
+        <v>11</v>
+      </c>
+      <c r="C69" t="s">
+        <v>49</v>
+      </c>
+      <c r="D69" t="s">
+        <v>82</v>
+      </c>
+      <c r="E69">
+        <v>48310</v>
+      </c>
+      <c r="F69" t="s">
+        <v>85</v>
+      </c>
+      <c r="G69" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7">
+      <c r="A70" t="s">
+        <v>7</v>
+      </c>
+      <c r="B70" t="s">
+        <v>11</v>
+      </c>
+      <c r="C70" t="s">
+        <v>49</v>
+      </c>
+      <c r="D70" t="s">
+        <v>82</v>
+      </c>
+      <c r="E70">
+        <v>48310</v>
+      </c>
+      <c r="F70" t="s">
+        <v>85</v>
+      </c>
+      <c r="G70" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7">
+      <c r="A71" t="s">
+        <v>7</v>
+      </c>
+      <c r="B71" t="s">
+        <v>11</v>
+      </c>
+      <c r="C71" t="s">
+        <v>49</v>
+      </c>
+      <c r="D71" t="s">
+        <v>82</v>
+      </c>
+      <c r="E71">
+        <v>48310</v>
+      </c>
+      <c r="F71" t="s">
+        <v>85</v>
+      </c>
+      <c r="G71" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7">
+      <c r="A72" t="s">
+        <v>7</v>
+      </c>
+      <c r="B72" t="s">
+        <v>11</v>
+      </c>
+      <c r="C72" t="s">
+        <v>50</v>
+      </c>
+      <c r="D72" t="s">
+        <v>82</v>
+      </c>
+      <c r="E72">
+        <v>48460</v>
+      </c>
+      <c r="F72" t="s">
+        <v>85</v>
+      </c>
+      <c r="G72" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7">
+      <c r="A73" t="s">
+        <v>7</v>
+      </c>
+      <c r="B73" t="s">
+        <v>11</v>
+      </c>
+      <c r="C73" t="s">
+        <v>50</v>
+      </c>
+      <c r="D73" t="s">
+        <v>82</v>
+      </c>
+      <c r="E73">
+        <v>48460</v>
+      </c>
+      <c r="F73" t="s">
+        <v>85</v>
+      </c>
+      <c r="G73" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7">
+      <c r="A74" t="s">
+        <v>7</v>
+      </c>
+      <c r="B74" t="s">
+        <v>11</v>
+      </c>
+      <c r="C74" t="s">
+        <v>50</v>
+      </c>
+      <c r="D74" t="s">
+        <v>82</v>
+      </c>
+      <c r="E74">
+        <v>48460</v>
+      </c>
+      <c r="F74" t="s">
+        <v>85</v>
+      </c>
+      <c r="G74" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7">
+      <c r="A75" t="s">
+        <v>7</v>
+      </c>
+      <c r="B75" t="s">
+        <v>11</v>
+      </c>
+      <c r="C75" t="s">
+        <v>51</v>
+      </c>
+      <c r="D75" t="s">
+        <v>83</v>
+      </c>
+      <c r="E75">
+        <v>49700</v>
+      </c>
+      <c r="F75" t="s">
+        <v>85</v>
+      </c>
+      <c r="G75" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7">
+      <c r="A76" t="s">
+        <v>7</v>
+      </c>
+      <c r="B76" t="s">
+        <v>11</v>
+      </c>
+      <c r="C76" t="s">
+        <v>51</v>
+      </c>
+      <c r="D76" t="s">
+        <v>83</v>
+      </c>
+      <c r="E76">
+        <v>49700</v>
+      </c>
+      <c r="F76" t="s">
+        <v>85</v>
+      </c>
+      <c r="G76" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7">
+      <c r="A77" t="s">
+        <v>7</v>
+      </c>
+      <c r="B77" t="s">
+        <v>11</v>
+      </c>
+      <c r="C77" t="s">
+        <v>51</v>
+      </c>
+      <c r="D77" t="s">
+        <v>83</v>
+      </c>
+      <c r="E77">
+        <v>49700</v>
+      </c>
+      <c r="F77" t="s">
+        <v>85</v>
+      </c>
+      <c r="G77" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7">
+      <c r="A78" t="s">
+        <v>7</v>
+      </c>
+      <c r="B78" t="s">
+        <v>11</v>
+      </c>
+      <c r="C78" t="s">
+        <v>52</v>
+      </c>
+      <c r="D78" t="s">
+        <v>83</v>
+      </c>
+      <c r="E78">
+        <v>51090</v>
+      </c>
+      <c r="F78" t="s">
+        <v>85</v>
+      </c>
+      <c r="G78" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7">
+      <c r="A79" t="s">
+        <v>7</v>
+      </c>
+      <c r="B79" t="s">
+        <v>11</v>
+      </c>
+      <c r="C79" t="s">
+        <v>52</v>
+      </c>
+      <c r="D79" t="s">
+        <v>83</v>
+      </c>
+      <c r="E79">
+        <v>51090</v>
+      </c>
+      <c r="F79" t="s">
+        <v>85</v>
+      </c>
+      <c r="G79" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7">
+      <c r="A80" t="s">
+        <v>7</v>
+      </c>
+      <c r="B80" t="s">
+        <v>11</v>
+      </c>
+      <c r="C80" t="s">
+        <v>52</v>
+      </c>
+      <c r="D80" t="s">
+        <v>83</v>
+      </c>
+      <c r="E80">
+        <v>51090</v>
+      </c>
+      <c r="F80" t="s">
+        <v>85</v>
+      </c>
+      <c r="G80" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7">
+      <c r="A81" t="s">
+        <v>7</v>
+      </c>
+      <c r="B81" t="s">
+        <v>11</v>
+      </c>
+      <c r="C81" t="s">
+        <v>53</v>
+      </c>
+      <c r="D81" t="s">
+        <v>83</v>
+      </c>
+      <c r="E81">
+        <v>52660</v>
+      </c>
+      <c r="F81" t="s">
+        <v>85</v>
+      </c>
+      <c r="G81" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7">
+      <c r="A82" t="s">
+        <v>7</v>
+      </c>
+      <c r="B82" t="s">
+        <v>11</v>
+      </c>
+      <c r="C82" t="s">
+        <v>53</v>
+      </c>
+      <c r="D82" t="s">
+        <v>83</v>
+      </c>
+      <c r="E82">
+        <v>52660</v>
+      </c>
+      <c r="F82" t="s">
+        <v>85</v>
+      </c>
+      <c r="G82" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7">
+      <c r="A83" t="s">
+        <v>7</v>
+      </c>
+      <c r="B83" t="s">
+        <v>11</v>
+      </c>
+      <c r="C83" t="s">
+        <v>53</v>
+      </c>
+      <c r="D83" t="s">
+        <v>83</v>
+      </c>
+      <c r="E83">
+        <v>52660</v>
+      </c>
+      <c r="F83" t="s">
+        <v>85</v>
+      </c>
+      <c r="G83" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7">
+      <c r="A84" t="s">
+        <v>7</v>
+      </c>
+      <c r="B84" t="s">
+        <v>11</v>
+      </c>
+      <c r="C84" t="s">
+        <v>54</v>
+      </c>
+      <c r="D84" t="s">
+        <v>84</v>
+      </c>
+      <c r="E84">
         <v>54740</v>
       </c>
-      <c r="F13" t="s">
-        <v>29</v>
-      </c>
-      <c r="G13" t="s">
-        <v>41</v>
+      <c r="F84" t="s">
+        <v>85</v>
+      </c>
+      <c r="G84" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7">
+      <c r="A85" t="s">
+        <v>7</v>
+      </c>
+      <c r="B85" t="s">
+        <v>11</v>
+      </c>
+      <c r="C85" t="s">
+        <v>54</v>
+      </c>
+      <c r="D85" t="s">
+        <v>84</v>
+      </c>
+      <c r="E85">
+        <v>54740</v>
+      </c>
+      <c r="F85" t="s">
+        <v>85</v>
+      </c>
+      <c r="G85" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7">
+      <c r="A86" t="s">
+        <v>7</v>
+      </c>
+      <c r="B86" t="s">
+        <v>11</v>
+      </c>
+      <c r="C86" t="s">
+        <v>54</v>
+      </c>
+      <c r="D86" t="s">
+        <v>84</v>
+      </c>
+      <c r="E86">
+        <v>54740</v>
+      </c>
+      <c r="F86" t="s">
+        <v>85</v>
+      </c>
+      <c r="G86" t="s">
+        <v>170</v>
       </c>
     </row>
   </sheetData>

</xml_diff>